<commit_message>
Align supplementary materials and documentation with revised manuscript
</commit_message>
<xml_diff>
--- a/supplementary-material/Supplementary Table S10.xlsx
+++ b/supplementary-material/Supplementary Table S10.xlsx
@@ -3,12 +3,17 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10404"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F9D1775-46EB-5C41-8B0A-DF6035A50BD1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/huhuiling/AI_Employment/4 paper：VR WCE/Supplement827/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF22CB17-A1F4-DB47-9AE4-35CD4ED27452}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="16240" yWindow="4960" windowWidth="15960" windowHeight="18080" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="15040" yWindow="5460" windowWidth="15960" windowHeight="18080" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="PCA90_K2" sheetId="1" r:id="rId1"/>
+    <sheet name="PCA90_K6" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
@@ -17,7 +22,7 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="94">
   <si>
-    <t>Sup6_PCA90 cluster_assignment_k2</t>
+    <t>PCA90 cluster assignments (K = 6)</t>
   </si>
   <si>
     <t>Video</t>
@@ -2409,7 +2414,7 @@
         <v>213.41069638259901</v>
       </c>
       <c r="CM3" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="CN3" s="5">
         <v>-1.15175905156082</v>
@@ -2690,7 +2695,7 @@
         <v>258.96999073371097</v>
       </c>
       <c r="CM4" s="11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="CN4" s="11">
         <v>-0.81886768990575598</v>
@@ -3252,7 +3257,7 @@
         <v>324.39653879142702</v>
       </c>
       <c r="CM6" s="11">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="CN6" s="11">
         <v>1.04942668762448</v>
@@ -3533,7 +3538,7 @@
         <v>223.07904834861699</v>
       </c>
       <c r="CM7" s="11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="CN7" s="11">
         <v>-3.1779413366794702</v>
@@ -3814,7 +3819,7 @@
         <v>227.25761750155999</v>
       </c>
       <c r="CM8" s="11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="CN8" s="11">
         <v>-4.3515530455607196</v>
@@ -4095,7 +4100,7 @@
         <v>258.34830589414503</v>
       </c>
       <c r="CM9" s="11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="CN9" s="11">
         <v>-0.99814487583955702</v>
@@ -4376,7 +4381,7 @@
         <v>259.18678862401902</v>
       </c>
       <c r="CM10" s="11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="CN10" s="11">
         <v>-1.23008833942106</v>
@@ -4657,7 +4662,7 @@
         <v>234.25770196004399</v>
       </c>
       <c r="CM11" s="11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="CN11" s="11">
         <v>-2.4949139206284898</v>
@@ -4938,7 +4943,7 @@
         <v>404.767702681591</v>
       </c>
       <c r="CM12" s="11">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="CN12" s="11">
         <v>8.2368964206116395</v>
@@ -5500,7 +5505,7 @@
         <v>226.65915358536299</v>
       </c>
       <c r="CM14" s="11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="CN14" s="11">
         <v>-0.99682847200713598</v>
@@ -6062,7 +6067,7 @@
         <v>233.205867343314</v>
       </c>
       <c r="CM16" s="11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="CN16" s="11">
         <v>-1.1825538774208999</v>
@@ -6343,7 +6348,7 @@
         <v>241.47161928907099</v>
       </c>
       <c r="CM17" s="11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="CN17" s="11">
         <v>-0.245133061510002</v>
@@ -6905,7 +6910,7 @@
         <v>240.14141372289299</v>
       </c>
       <c r="CM19" s="11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="CN19" s="11">
         <v>-1.5713076519320099</v>
@@ -7186,7 +7191,7 @@
         <v>242.11129408405799</v>
       </c>
       <c r="CM20" s="11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="CN20" s="11">
         <v>-1.79353813836995</v>
@@ -7467,7 +7472,7 @@
         <v>179.603098360616</v>
       </c>
       <c r="CM21" s="11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="CN21" s="11">
         <v>-4.8473486123587</v>
@@ -7748,7 +7753,7 @@
         <v>204.21536461042999</v>
       </c>
       <c r="CM22" s="11">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="CN22" s="11">
         <v>-7.3837218372907598</v>
@@ -8029,7 +8034,7 @@
         <v>240.15994142902201</v>
       </c>
       <c r="CM23" s="11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="CN23" s="11">
         <v>-2.3542352658748502</v>
@@ -8310,7 +8315,7 @@
         <v>215.96824673805699</v>
       </c>
       <c r="CM24" s="11">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="CN24" s="11">
         <v>-5.1539199562215297</v>
@@ -8591,7 +8596,7 @@
         <v>215.36167927653599</v>
       </c>
       <c r="CM25" s="11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="CN25" s="11">
         <v>-2.85143979751179</v>
@@ -8872,7 +8877,7 @@
         <v>191.244646363946</v>
       </c>
       <c r="CM26" s="11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="CN26" s="11">
         <v>-3.3131252177071402</v>
@@ -9153,7 +9158,7 @@
         <v>222.71798655167001</v>
       </c>
       <c r="CM27" s="11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="CN27" s="11">
         <v>-1.6279802634659899</v>
@@ -9996,7 +10001,7 @@
         <v>250.46400960631999</v>
       </c>
       <c r="CM30" s="11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="CN30" s="11">
         <v>-0.18561918157003701</v>
@@ -10558,7 +10563,7 @@
         <v>215.75120247357501</v>
       </c>
       <c r="CM32" s="11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="CN32" s="11">
         <v>-0.94936033286453003</v>
@@ -11120,7 +11125,7 @@
         <v>264.43903713777797</v>
       </c>
       <c r="CM34" s="11">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="CN34" s="11">
         <v>2.99472578065483</v>
@@ -11401,7 +11406,7 @@
         <v>307.84161372863201</v>
       </c>
       <c r="CM35" s="11">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="CN35" s="11">
         <v>5.4365293463536402</v>
@@ -11682,7 +11687,7 @@
         <v>359.38051532047598</v>
       </c>
       <c r="CM36" s="11">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="CN36" s="11">
         <v>7.5995654407353097</v>
@@ -11963,7 +11968,7 @@
         <v>341.78863439531102</v>
       </c>
       <c r="CM37" s="11">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="CN37" s="11">
         <v>3.9406354529138601</v>
@@ -12244,7 +12249,7 @@
         <v>430.24172349243702</v>
       </c>
       <c r="CM38" s="11">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="CN38" s="11">
         <v>8.1156664184498801</v>
@@ -12525,7 +12530,7 @@
         <v>390.21290259761702</v>
       </c>
       <c r="CM39" s="11">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="CN39" s="11">
         <v>6.8865985118173603</v>
@@ -12806,7 +12811,7 @@
         <v>414.02285944137498</v>
       </c>
       <c r="CM40" s="11">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="CN40" s="11">
         <v>7.5555863170117403</v>
@@ -13087,7 +13092,7 @@
         <v>433.50878977690701</v>
       </c>
       <c r="CM41" s="11">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="CN41" s="11">
         <v>9.5604591084231991</v>
@@ -13368,7 +13373,7 @@
         <v>439.90501294623402</v>
       </c>
       <c r="CM42" s="11">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="CN42" s="11">
         <v>11.7358738676628</v>
@@ -13649,7 +13654,7 @@
         <v>405.76444039137402</v>
       </c>
       <c r="CM43" s="11">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="CN43" s="11">
         <v>10.4434026467487</v>
@@ -13930,7 +13935,7 @@
         <v>596.443076772979</v>
       </c>
       <c r="CM44" s="11">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="CN44" s="11">
         <v>25.128668604595902</v>
@@ -14211,7 +14216,7 @@
         <v>460.93889228118701</v>
       </c>
       <c r="CM45" s="11">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="CN45" s="11">
         <v>18.022721733446701</v>
@@ -14492,7 +14497,7 @@
         <v>487.096326208638</v>
       </c>
       <c r="CM46" s="11">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="CN46" s="11">
         <v>18.0691277394499</v>
@@ -14773,7 +14778,7 @@
         <v>518.39037428493498</v>
       </c>
       <c r="CM47" s="11">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="CN47" s="11">
         <v>19.163684857301899</v>
@@ -15054,7 +15059,7 @@
         <v>394.80570602248002</v>
       </c>
       <c r="CM48" s="11">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="CN48" s="11">
         <v>6.5152426014501801</v>
@@ -15335,7 +15340,7 @@
         <v>343.57517593925502</v>
       </c>
       <c r="CM49" s="11">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="CN49" s="11">
         <v>5.2811310366538899</v>
@@ -15616,7 +15621,7 @@
         <v>417.23686956629399</v>
       </c>
       <c r="CM50" s="11">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="CN50" s="11">
         <v>7.0871939437495497</v>
@@ -15897,7 +15902,7 @@
         <v>323.38520438090501</v>
       </c>
       <c r="CM51" s="11">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="CN51" s="11">
         <v>4.7160880136773802</v>
@@ -16178,7 +16183,7 @@
         <v>377.67435088882598</v>
       </c>
       <c r="CM52" s="11">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="CN52" s="11">
         <v>5.9914095018106401</v>
@@ -16459,7 +16464,7 @@
         <v>479.87541405242501</v>
       </c>
       <c r="CM53" s="11">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="CN53" s="11">
         <v>12.8190591663499</v>
@@ -16740,7 +16745,7 @@
         <v>461.90650107675702</v>
       </c>
       <c r="CM54" s="11">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="CN54" s="11">
         <v>12.736282967645799</v>
@@ -17021,7 +17026,7 @@
         <v>491.484249196848</v>
       </c>
       <c r="CM55" s="11">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="CN55" s="11">
         <v>12.791227744083599</v>
@@ -17302,7 +17307,7 @@
         <v>496.66021690487003</v>
       </c>
       <c r="CM56" s="11">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="CN56" s="11">
         <v>16.5453756492766</v>
@@ -17583,7 +17588,7 @@
         <v>521.22433385048305</v>
       </c>
       <c r="CM57" s="11">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="CN57" s="11">
         <v>16.7591865445265</v>
@@ -17864,7 +17869,7 @@
         <v>470.61151074895901</v>
       </c>
       <c r="CM58" s="11">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="CN58" s="11">
         <v>12.9948279240079</v>
@@ -18145,7 +18150,7 @@
         <v>451.21990895472902</v>
       </c>
       <c r="CM59" s="11">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="CN59" s="11">
         <v>12.332553751362299</v>
@@ -18426,7 +18431,7 @@
         <v>423.69105700707502</v>
       </c>
       <c r="CM60" s="11">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="CN60" s="11">
         <v>10.0624750852006</v>
@@ -18707,7 +18712,7 @@
         <v>447.40121068970001</v>
       </c>
       <c r="CM61" s="11">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="CN61" s="11">
         <v>11.028968816714301</v>
@@ -18988,7 +18993,7 @@
         <v>395.92388531048903</v>
       </c>
       <c r="CM62" s="11">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="CN62" s="11">
         <v>7.6905464722126498</v>
@@ -19269,7 +19274,7 @@
         <v>425.309597925128</v>
       </c>
       <c r="CM63" s="11">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="CN63" s="11">
         <v>9.2713619326209695</v>
@@ -19550,7 +19555,7 @@
         <v>371.720493862696</v>
       </c>
       <c r="CM64" s="11">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="CN64" s="11">
         <v>4.9706481120901698</v>
@@ -19831,7 +19836,7 @@
         <v>383.57325192507</v>
       </c>
       <c r="CM65" s="11">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="CN65" s="11">
         <v>7.28152798412781</v>
@@ -20112,7 +20117,7 @@
         <v>293.16481299216798</v>
       </c>
       <c r="CM66" s="11">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="CN66" s="11">
         <v>0.75468785256744497</v>
@@ -20393,7 +20398,7 @@
         <v>332.54884715319997</v>
       </c>
       <c r="CM67" s="11">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="CN67" s="11">
         <v>3.4421019163527999</v>
@@ -20674,7 +20679,7 @@
         <v>267.711893142397</v>
       </c>
       <c r="CM68" s="11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="CN68" s="11">
         <v>-1.4068207178784</v>
@@ -20955,7 +20960,7 @@
         <v>258.90322416858402</v>
       </c>
       <c r="CM69" s="11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="CN69" s="11">
         <v>-0.92753935140272203</v>
@@ -21236,7 +21241,7 @@
         <v>285.97578549357002</v>
       </c>
       <c r="CM70" s="11">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="CN70" s="11">
         <v>3.2289629430627702</v>
@@ -21517,7 +21522,7 @@
         <v>216.54972640879001</v>
       </c>
       <c r="CM71" s="11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="CN71" s="11">
         <v>-2.27925041767514</v>
@@ -21798,7 +21803,7 @@
         <v>242.262185626182</v>
       </c>
       <c r="CM72" s="11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="CN72" s="11">
         <v>-2.2991368185969701</v>
@@ -22079,7 +22084,7 @@
         <v>306.06589229850903</v>
       </c>
       <c r="CM73" s="11">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="CN73" s="11">
         <v>7.2279656253312501</v>
@@ -22360,7 +22365,7 @@
         <v>304.40361316142503</v>
       </c>
       <c r="CM74" s="11">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="CN74" s="11">
         <v>1.44761328659052</v>
@@ -22641,7 +22646,7 @@
         <v>391.26579614426299</v>
       </c>
       <c r="CM75" s="11">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="CN75" s="11">
         <v>8.7301969669288706</v>
@@ -22922,7 +22927,7 @@
         <v>385.53564542104698</v>
       </c>
       <c r="CM76" s="11">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="CN76" s="11">
         <v>5.9554038441483703</v>
@@ -23203,7 +23208,7 @@
         <v>433.12915831484497</v>
       </c>
       <c r="CM77" s="11">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="CN77" s="11">
         <v>7.7780027937315204</v>
@@ -23484,7 +23489,7 @@
         <v>363.75010025197003</v>
       </c>
       <c r="CM78" s="11">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="CN78" s="11">
         <v>4.5789857031289003</v>
@@ -23765,7 +23770,7 @@
         <v>460.76105381886299</v>
       </c>
       <c r="CM79" s="11">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="CN79" s="11">
         <v>11.5826236839172</v>
@@ -24046,7 +24051,7 @@
         <v>404.69322231225902</v>
       </c>
       <c r="CM80" s="11">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="CN80" s="11">
         <v>6.5348357775823001</v>
@@ -24327,7 +24332,7 @@
         <v>355.06177716800698</v>
       </c>
       <c r="CM81" s="11">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="CN81" s="11">
         <v>5.2885843299571</v>
@@ -24608,7 +24613,7 @@
         <v>398.15255981245002</v>
       </c>
       <c r="CM82" s="11">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="CN82" s="11">
         <v>6.7614572226096996</v>
@@ -24889,7 +24894,7 @@
         <v>303.783894027261</v>
       </c>
       <c r="CM83" s="11">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="CN83" s="11">
         <v>1.33743769545639</v>
@@ -25170,7 +25175,7 @@
         <v>323.39344134466302</v>
       </c>
       <c r="CM84" s="11">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="CN84" s="11">
         <v>2.4500666030899501</v>
@@ -25451,7 +25456,7 @@
         <v>322.25847975145899</v>
       </c>
       <c r="CM85" s="11">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="CN85" s="11">
         <v>2.0189536378662098</v>
@@ -25732,7 +25737,7 @@
         <v>335.69264831415899</v>
       </c>
       <c r="CM86" s="11">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="CN86" s="11">
         <v>4.0489214237598103</v>
@@ -26013,7 +26018,7 @@
         <v>344.21818547375301</v>
       </c>
       <c r="CM87" s="11">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="CN87" s="11">
         <v>2.8165372496594498</v>
@@ -26294,7 +26299,7 @@
         <v>299.24530385219703</v>
       </c>
       <c r="CM88" s="11">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="CN88" s="11">
         <v>5.0932860593332299</v>
@@ -26575,7 +26580,7 @@
         <v>276.74216632577998</v>
       </c>
       <c r="CM89" s="11">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="CN89" s="11">
         <v>2.5525616157983499</v>
@@ -26856,7 +26861,7 @@
         <v>304.028587991677</v>
       </c>
       <c r="CM90" s="11">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="CN90" s="11">
         <v>4.6830700737470199</v>
@@ -27137,7 +27142,7 @@
         <v>330.01920685761598</v>
       </c>
       <c r="CM91" s="11">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="CN91" s="11">
         <v>3.5693510982848098</v>
@@ -27418,7 +27423,7 @@
         <v>267.93633666107303</v>
       </c>
       <c r="CM92" s="11">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="CN92" s="11">
         <v>2.8482294355325202</v>
@@ -27699,7 +27704,7 @@
         <v>251.8636744918</v>
       </c>
       <c r="CM93" s="11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="CN93" s="11">
         <v>-2.0951524186703101</v>
@@ -28542,7 +28547,7 @@
         <v>251.89850086853801</v>
       </c>
       <c r="CM96" s="11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="CN96" s="11">
         <v>-0.95702223657444296</v>
@@ -28823,7 +28828,7 @@
         <v>303.79813584662202</v>
       </c>
       <c r="CM97" s="11">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="CN97" s="11">
         <v>1.2841602651393</v>
@@ -29104,7 +29109,7 @@
         <v>232.54833262279999</v>
       </c>
       <c r="CM98" s="11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="CN98" s="11">
         <v>-3.58134970997757</v>
@@ -29385,7 +29390,7 @@
         <v>240.72011948420899</v>
       </c>
       <c r="CM99" s="11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="CN99" s="11">
         <v>-3.6721269538841201</v>
@@ -29666,7 +29671,7 @@
         <v>237.48682573476199</v>
       </c>
       <c r="CM100" s="11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="CN100" s="11">
         <v>-4.6039845808978699</v>
@@ -29947,7 +29952,7 @@
         <v>312.59434514833902</v>
       </c>
       <c r="CM101" s="11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="CN101" s="11">
         <v>-0.52645557961558298</v>
@@ -30228,7 +30233,7 @@
         <v>212.62307707923901</v>
       </c>
       <c r="CM102" s="11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="CN102" s="11">
         <v>-3.7952224703517201</v>
@@ -30509,7 +30514,7 @@
         <v>316.42780907954301</v>
       </c>
       <c r="CM103" s="11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="CN103" s="11">
         <v>-0.20892875612829701</v>
@@ -31914,7 +31919,7 @@
         <v>225.64176413079599</v>
       </c>
       <c r="CM108" s="11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="CN108" s="11">
         <v>-2.88218385802507</v>
@@ -32195,7 +32200,7 @@
         <v>246.41598376442499</v>
       </c>
       <c r="CM109" s="11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="CN109" s="11">
         <v>-1.1771009475033001</v>
@@ -32476,7 +32481,7 @@
         <v>244.90762466657699</v>
       </c>
       <c r="CM110" s="11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="CN110" s="11">
         <v>-1.76020681173533</v>
@@ -32757,7 +32762,7 @@
         <v>258.66837626881301</v>
       </c>
       <c r="CM111" s="11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="CN111" s="11">
         <v>-2.0640541598717799</v>
@@ -33038,7 +33043,7 @@
         <v>370.736104869033</v>
       </c>
       <c r="CM112" s="11">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="CN112" s="11">
         <v>7.6531500140499196</v>
@@ -33319,7 +33324,7 @@
         <v>269.19513275367899</v>
       </c>
       <c r="CM113" s="11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="CN113" s="11">
         <v>-1.5715153586588599</v>
@@ -33600,7 +33605,7 @@
         <v>266.17421121294001</v>
       </c>
       <c r="CM114" s="11">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="CN114" s="11">
         <v>3.4549077632094298</v>
@@ -33881,7 +33886,7 @@
         <v>242.26152096890399</v>
       </c>
       <c r="CM115" s="11">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="CN115" s="11">
         <v>0.76856504478008603</v>
@@ -34162,7 +34167,7 @@
         <v>332.93642904301998</v>
       </c>
       <c r="CM116" s="11">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="CN116" s="11">
         <v>4.6531796274851702</v>
@@ -34443,7 +34448,7 @@
         <v>363.60021838463501</v>
       </c>
       <c r="CM117" s="11">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="CN117" s="11">
         <v>7.41266904525264</v>
@@ -34724,7 +34729,7 @@
         <v>287.67492504835201</v>
       </c>
       <c r="CM118" s="11">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="CN118" s="11">
         <v>1.80067826348536</v>
@@ -35005,7 +35010,7 @@
         <v>269.50445634897801</v>
       </c>
       <c r="CM119" s="11">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="CN119" s="11">
         <v>1.01903823986219</v>
@@ -35567,7 +35572,7 @@
         <v>256.36832661452098</v>
       </c>
       <c r="CM121" s="11">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="CN121" s="11">
         <v>0.48516591748832599</v>
@@ -35848,7 +35853,7 @@
         <v>287.93748679054198</v>
       </c>
       <c r="CM122" s="11">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="CN122" s="11">
         <v>3.4754522460541999</v>
@@ -36129,7 +36134,7 @@
         <v>263.44977187377401</v>
       </c>
       <c r="CM123" s="11">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="CN123" s="11">
         <v>1.82371703808956</v>
@@ -36410,7 +36415,7 @@
         <v>265.729152554834</v>
       </c>
       <c r="CM124" s="11">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="CN124" s="11">
         <v>2.8128621171050399</v>
@@ -36691,7 +36696,7 @@
         <v>271.74677750647402</v>
       </c>
       <c r="CM125" s="11">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="CN125" s="11">
         <v>2.645249054212</v>
@@ -36972,7 +36977,7 @@
         <v>277.02892362474199</v>
       </c>
       <c r="CM126" s="11">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="CN126" s="11">
         <v>5.92776084570073</v>
@@ -37253,7 +37258,7 @@
         <v>329.46767755752398</v>
       </c>
       <c r="CM127" s="11">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="CN127" s="11">
         <v>-0.476605307999246</v>
@@ -37534,7 +37539,7 @@
         <v>406.67222920898098</v>
       </c>
       <c r="CM128" s="11">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="CN128" s="11">
         <v>8.6018354776617603</v>
@@ -37815,7 +37820,7 @@
         <v>281.19679773643099</v>
       </c>
       <c r="CM129" s="11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="CN129" s="11">
         <v>-1.8648916660477299</v>
@@ -38096,7 +38101,7 @@
         <v>274.827574159562</v>
       </c>
       <c r="CM130" s="11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="CN130" s="11">
         <v>-2.7664732081228798</v>
@@ -38377,7 +38382,7 @@
         <v>378.07360076234301</v>
       </c>
       <c r="CM131" s="11">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="CN131" s="11">
         <v>4.5372159387775</v>
@@ -38658,7 +38663,7 @@
         <v>316.40983900103902</v>
       </c>
       <c r="CM132" s="11">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="CN132" s="11">
         <v>1.7880169265458501</v>
@@ -38939,7 +38944,7 @@
         <v>339.19126883442999</v>
       </c>
       <c r="CM133" s="11">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="CN133" s="11">
         <v>2.13657164418913</v>
@@ -39220,7 +39225,7 @@
         <v>326.908459815843</v>
       </c>
       <c r="CM134" s="11">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="CN134" s="11">
         <v>2.7032773935679302</v>
@@ -39501,7 +39506,7 @@
         <v>329.07509631047299</v>
       </c>
       <c r="CM135" s="11">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="CN135" s="11">
         <v>3.2228630106343501</v>
@@ -39782,7 +39787,7 @@
         <v>441.80685580565103</v>
       </c>
       <c r="CM136" s="11">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="CN136" s="11">
         <v>9.5520826729684298</v>
@@ -40063,7 +40068,7 @@
         <v>371.27211701056399</v>
       </c>
       <c r="CM137" s="11">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="CN137" s="11">
         <v>4.4424063121816104</v>
@@ -40344,7 +40349,7 @@
         <v>346.92565315210999</v>
       </c>
       <c r="CM138" s="11">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="CN138" s="11">
         <v>3.9260384813459899</v>
@@ -40625,7 +40630,7 @@
         <v>344.40866622785097</v>
       </c>
       <c r="CM139" s="11">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="CN139" s="11">
         <v>3.8808106864941401</v>
@@ -40906,7 +40911,7 @@
         <v>348.82663539441103</v>
       </c>
       <c r="CM140" s="11">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="CN140" s="11">
         <v>3.3782314458978302</v>
@@ -41187,7 +41192,7 @@
         <v>316.97842203258199</v>
       </c>
       <c r="CM141" s="11">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="CN141" s="11">
         <v>2.04361597654903</v>
@@ -41468,7 +41473,7 @@
         <v>359.92324288358299</v>
       </c>
       <c r="CM142" s="11">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="CN142" s="11">
         <v>5.8306021578420602</v>
@@ -41749,7 +41754,7 @@
         <v>296.73624371848302</v>
       </c>
       <c r="CM143" s="11">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="CN143" s="11">
         <v>2.6500171961455901</v>
@@ -42030,7 +42035,7 @@
         <v>356.81458265785801</v>
       </c>
       <c r="CM144" s="11">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="CN144" s="11">
         <v>1.51646110878961</v>
@@ -42311,7 +42316,7 @@
         <v>356.88653598302801</v>
       </c>
       <c r="CM145" s="11">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="CN145" s="11">
         <v>4.2890218290713502</v>
@@ -42592,7 +42597,7 @@
         <v>274.16294093125799</v>
       </c>
       <c r="CM146" s="11">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="CN146" s="11">
         <v>1.1920543753548301</v>
@@ -42873,7 +42878,7 @@
         <v>314.98740553754197</v>
       </c>
       <c r="CM147" s="11">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="CN147" s="11">
         <v>3.93581238295058</v>
@@ -43154,7 +43159,7 @@
         <v>400.09700488016802</v>
       </c>
       <c r="CM148" s="11">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="CN148" s="11">
         <v>6.8357910976174399</v>
@@ -43435,7 +43440,7 @@
         <v>293.156265471545</v>
       </c>
       <c r="CM149" s="11">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="CN149" s="11">
         <v>-0.49308298831987601</v>
@@ -43716,7 +43721,7 @@
         <v>407.52297833466002</v>
       </c>
       <c r="CM150" s="11">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="CN150" s="11">
         <v>7.4269800604068603</v>
@@ -43997,7 +44002,7 @@
         <v>384.995511592855</v>
       </c>
       <c r="CM151" s="11">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="CN151" s="11">
         <v>7.7728791108374802</v>
@@ -44278,7 +44283,7 @@
         <v>336.22915272800202</v>
       </c>
       <c r="CM152" s="11">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="CN152" s="11">
         <v>8.4180653139198096</v>
@@ -44559,7 +44564,7 @@
         <v>321.08787971577198</v>
       </c>
       <c r="CM153" s="11">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="CN153" s="11">
         <v>5.00534817752348</v>
@@ -44840,7 +44845,7 @@
         <v>376.34674530899701</v>
       </c>
       <c r="CM154" s="11">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="CN154" s="11">
         <v>5.6167278949727102</v>
@@ -45121,7 +45126,7 @@
         <v>331.86023744212901</v>
       </c>
       <c r="CM155" s="11">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="CN155" s="11">
         <v>3.4130758019106602</v>
@@ -45402,7 +45407,7 @@
         <v>351.90880999290198</v>
       </c>
       <c r="CM156" s="11">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="CN156" s="11">
         <v>3.1164724389234402</v>
@@ -45683,7 +45688,7 @@
         <v>338.14954279242698</v>
       </c>
       <c r="CM157" s="11">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="CN157" s="11">
         <v>2.4804053990378998</v>
@@ -45964,7 +45969,7 @@
         <v>336.39742782675302</v>
       </c>
       <c r="CM158" s="11">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="CN158" s="11">
         <v>2.7943899117548199</v>
@@ -46245,7 +46250,7 @@
         <v>337.559917945824</v>
       </c>
       <c r="CM159" s="11">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="CN159" s="11">
         <v>4.3868495526188704</v>
@@ -46526,7 +46531,7 @@
         <v>353.684342207074</v>
       </c>
       <c r="CM160" s="11">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="CN160" s="11">
         <v>4.4522266629090099</v>
@@ -46807,7 +46812,7 @@
         <v>354.43657347912898</v>
       </c>
       <c r="CM161" s="11">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="CN161" s="11">
         <v>6.05117199751363</v>
@@ -47088,7 +47093,7 @@
         <v>346.315888515621</v>
       </c>
       <c r="CM162" s="11">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="CN162" s="11">
         <v>1.8446282171733199</v>
@@ -47369,7 +47374,7 @@
         <v>361.38850589001999</v>
       </c>
       <c r="CM163" s="11">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="CN163" s="11">
         <v>6.0807075601774798</v>
@@ -47650,7 +47655,7 @@
         <v>380.43367621545502</v>
       </c>
       <c r="CM164" s="11">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="CN164" s="11">
         <v>5.3830156651596104</v>
@@ -47931,7 +47936,7 @@
         <v>352.54921595998599</v>
       </c>
       <c r="CM165" s="11">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="CN165" s="11">
         <v>1.9021929924716601</v>
@@ -48212,7 +48217,7 @@
         <v>343.628304223312</v>
       </c>
       <c r="CM166" s="11">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="CN166" s="11">
         <v>3.6724902713102798</v>
@@ -48493,7 +48498,7 @@
         <v>365.63690682400397</v>
       </c>
       <c r="CM167" s="11">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="CN167" s="11">
         <v>3.4862181009014401</v>
@@ -48774,7 +48779,7 @@
         <v>383.09006298638599</v>
       </c>
       <c r="CM168" s="11">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="CN168" s="11">
         <v>4.90317092604697</v>
@@ -49055,7 +49060,7 @@
         <v>140.794454774305</v>
       </c>
       <c r="CM169" s="11">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="CN169" s="11">
         <v>-7.7182166630019502</v>
@@ -49336,7 +49341,7 @@
         <v>181.11404741981201</v>
       </c>
       <c r="CM170" s="11">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="CN170" s="11">
         <v>-6.3917700081679403</v>
@@ -49617,7 +49622,7 @@
         <v>216.386068251577</v>
       </c>
       <c r="CM171" s="11">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="CN171" s="11">
         <v>-4.8113260078701501</v>
@@ -49898,7 +49903,7 @@
         <v>134.429556212085</v>
       </c>
       <c r="CM172" s="11">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="CN172" s="11">
         <v>-11.8467365378295</v>
@@ -50179,7 +50184,7 @@
         <v>124.755208814223</v>
       </c>
       <c r="CM173" s="11">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="CN173" s="11">
         <v>-12.423847321282601</v>
@@ -50460,7 +50465,7 @@
         <v>90.025251163846903</v>
       </c>
       <c r="CM174" s="11">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="CN174" s="11">
         <v>-12.2871082384075</v>
@@ -50741,7 +50746,7 @@
         <v>117.608996851257</v>
       </c>
       <c r="CM175" s="11">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="CN175" s="11">
         <v>-12.3346767438667</v>
@@ -51022,7 +51027,7 @@
         <v>90.782482158795204</v>
       </c>
       <c r="CM176" s="11">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="CN176" s="11">
         <v>-12.867248609982701</v>
@@ -51303,7 +51308,7 @@
         <v>154.34186546901199</v>
       </c>
       <c r="CM177" s="11">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="CN177" s="11">
         <v>-8.6918276282799898</v>
@@ -51584,7 +51589,7 @@
         <v>116.411920706499</v>
       </c>
       <c r="CM178" s="11">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="CN178" s="11">
         <v>-10.315244123777299</v>
@@ -51865,7 +51870,7 @@
         <v>142.810233282605</v>
       </c>
       <c r="CM179" s="11">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="CN179" s="11">
         <v>-9.6092170353789701</v>
@@ -52146,7 +52151,7 @@
         <v>113.395065912174</v>
       </c>
       <c r="CM180" s="11">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="CN180" s="11">
         <v>-10.986262201913499</v>
@@ -52427,7 +52432,7 @@
         <v>119.474969583488</v>
       </c>
       <c r="CM181" s="11">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="CN181" s="11">
         <v>-9.9201336085662604</v>
@@ -52708,7 +52713,7 @@
         <v>126.26738286625699</v>
       </c>
       <c r="CM182" s="11">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="CN182" s="11">
         <v>-9.7896581454865892</v>
@@ -52989,7 +52994,7 @@
         <v>200.73488477100301</v>
       </c>
       <c r="CM183" s="11">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="CN183" s="11">
         <v>-6.9241890198796598</v>
@@ -53270,7 +53275,7 @@
         <v>184.67723554853001</v>
       </c>
       <c r="CM184" s="11">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="CN184" s="11">
         <v>-10.813777817058201</v>
@@ -53551,7 +53556,7 @@
         <v>196.45551121552199</v>
       </c>
       <c r="CM185" s="11">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="CN185" s="11">
         <v>-9.2813203200971408</v>
@@ -53832,7 +53837,7 @@
         <v>281.85964030864398</v>
       </c>
       <c r="CM186" s="11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="CN186" s="11">
         <v>-0.38013872237125101</v>
@@ -54113,7 +54118,7 @@
         <v>110.391742670773</v>
       </c>
       <c r="CM187" s="11">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="CN187" s="11">
         <v>-14.0468729220781</v>
@@ -54394,7 +54399,7 @@
         <v>243.70124977123999</v>
       </c>
       <c r="CM188" s="11">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="CN188" s="11">
         <v>-4.9171413746360404</v>
@@ -54675,7 +54680,7 @@
         <v>146.388636359993</v>
       </c>
       <c r="CM189" s="11">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="CN189" s="11">
         <v>-12.1252209581485</v>
@@ -54956,7 +54961,7 @@
         <v>146.33513347908601</v>
       </c>
       <c r="CM190" s="11">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="CN190" s="11">
         <v>-11.467107380775699</v>
@@ -55237,7 +55242,7 @@
         <v>182.38478459678501</v>
       </c>
       <c r="CM191" s="11">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="CN191" s="11">
         <v>-8.9500505436208293</v>
@@ -55518,7 +55523,7 @@
         <v>167.642149939501</v>
       </c>
       <c r="CM192" s="11">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="CN192" s="11">
         <v>-10.8514893123719</v>
@@ -55799,7 +55804,7 @@
         <v>147.17322487946501</v>
       </c>
       <c r="CM193" s="11">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="CN193" s="11">
         <v>-11.148008081404001</v>
@@ -56080,7 +56085,7 @@
         <v>162.22874180662299</v>
       </c>
       <c r="CM194" s="11">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="CN194" s="11">
         <v>-10.298259026611699</v>
@@ -56361,7 +56366,7 @@
         <v>124.922980939124</v>
       </c>
       <c r="CM195" s="11">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="CN195" s="11">
         <v>-12.6230716569415</v>
@@ -56642,7 +56647,7 @@
         <v>171.56120394484699</v>
       </c>
       <c r="CM196" s="11">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="CN196" s="11">
         <v>-8.9607284865612709</v>
@@ -56923,7 +56928,7 @@
         <v>133.76305153000601</v>
       </c>
       <c r="CM197" s="11">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="CN197" s="11">
         <v>-11.506017636932899</v>
@@ -57204,7 +57209,7 @@
         <v>132.12907722094701</v>
       </c>
       <c r="CM198" s="11">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="CN198" s="11">
         <v>-9.0129389404752001</v>
@@ -57485,7 +57490,7 @@
         <v>145.73804506175699</v>
       </c>
       <c r="CM199" s="11">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="CN199" s="11">
         <v>-10.306658783363</v>
@@ -57766,7 +57771,7 @@
         <v>247.92309851899199</v>
       </c>
       <c r="CM200" s="11">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="CN200" s="11">
         <v>-5.55411884193001</v>
@@ -58047,7 +58052,7 @@
         <v>166.50099888200899</v>
       </c>
       <c r="CM201" s="11">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="CN201" s="11">
         <v>-8.5676083222147597</v>
@@ -58328,7 +58333,7 @@
         <v>150.81128801188299</v>
       </c>
       <c r="CM202" s="11">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="CN202" s="11">
         <v>-8.9464049050703007</v>
@@ -58609,7 +58614,7 @@
         <v>180.460265918891</v>
       </c>
       <c r="CM203" s="11">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="CN203" s="11">
         <v>-8.5608993540803109</v>
@@ -58890,7 +58895,7 @@
         <v>274.21850514528398</v>
       </c>
       <c r="CM204" s="11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="CN204" s="11">
         <v>-3.9203443645166902</v>
@@ -59171,7 +59176,7 @@
         <v>226.31648695815201</v>
       </c>
       <c r="CM205" s="11">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="CN205" s="11">
         <v>-5.4154631936434496</v>
@@ -59452,7 +59457,7 @@
         <v>252.962781277978</v>
       </c>
       <c r="CM206" s="11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="CN206" s="11">
         <v>-4.9081306707342902</v>
@@ -59733,7 +59738,7 @@
         <v>214.84428586128999</v>
       </c>
       <c r="CM207" s="11">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="CN207" s="11">
         <v>-9.2845106557853097</v>
@@ -60014,7 +60019,7 @@
         <v>200.977649403931</v>
       </c>
       <c r="CM208" s="11">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="CN208" s="11">
         <v>-6.0780971049246997</v>
@@ -60295,7 +60300,7 @@
         <v>228.79586799520101</v>
       </c>
       <c r="CM209" s="11">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="CN209" s="11">
         <v>-7.8369973663233399</v>
@@ -60576,7 +60581,7 @@
         <v>219.171867542775</v>
       </c>
       <c r="CM210" s="11">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="CN210" s="11">
         <v>-7.5359140236365798</v>
@@ -60857,7 +60862,7 @@
         <v>224.060488835336</v>
       </c>
       <c r="CM211" s="11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="CN211" s="11">
         <v>-3.2165418550804299</v>
@@ -61138,7 +61143,7 @@
         <v>231.04934593039999</v>
       </c>
       <c r="CM212" s="11">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="CN212" s="11">
         <v>-7.4452637137441702</v>
@@ -61419,7 +61424,7 @@
         <v>209.98442527515999</v>
       </c>
       <c r="CM213" s="11">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="CN213" s="11">
         <v>-5.58246116611285</v>
@@ -61700,7 +61705,7 @@
         <v>169.02715539226199</v>
       </c>
       <c r="CM214" s="11">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="CN214" s="11">
         <v>-7.8575830393644202</v>
@@ -61981,7 +61986,7 @@
         <v>258.38868070695497</v>
       </c>
       <c r="CM215" s="11">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="CN215" s="11">
         <v>-5.8973810912664604</v>
@@ -62262,7 +62267,7 @@
         <v>208.28383508721001</v>
       </c>
       <c r="CM216" s="11">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="CN216" s="11">
         <v>-7.8415245760208601</v>
@@ -62543,7 +62548,7 @@
         <v>187.86613670089099</v>
       </c>
       <c r="CM217" s="11">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="CN217" s="11">
         <v>-9.2874692797117095</v>
@@ -62824,7 +62829,7 @@
         <v>245.832717241696</v>
       </c>
       <c r="CM218" s="11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="CN218" s="11">
         <v>-5.0545368431418298</v>
@@ -63105,7 +63110,7 @@
         <v>206.12117192498201</v>
       </c>
       <c r="CM219" s="11">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="CN219" s="11">
         <v>-7.76185575899716</v>
@@ -63386,7 +63391,7 @@
         <v>252.842982403664</v>
       </c>
       <c r="CM220" s="11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="CN220" s="11">
         <v>-2.2149874287515501</v>
@@ -63667,7 +63672,7 @@
         <v>287.419477886143</v>
       </c>
       <c r="CM221" s="11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="CN221" s="11">
         <v>-2.3189010678647102</v>
@@ -63948,7 +63953,7 @@
         <v>200.89645058252199</v>
       </c>
       <c r="CM222" s="11">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="CN222" s="11">
         <v>-9.2816264755503504</v>
@@ -64229,7 +64234,7 @@
         <v>189.35956251586001</v>
       </c>
       <c r="CM223" s="11">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="CN223" s="11">
         <v>-9.1294216945008593</v>
@@ -64510,7 +64515,7 @@
         <v>196.53602567100199</v>
       </c>
       <c r="CM224" s="11">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="CN224" s="11">
         <v>-7.4123816512486496</v>
@@ -64791,7 +64796,7 @@
         <v>232.31597999239099</v>
       </c>
       <c r="CM225" s="11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="CN225" s="11">
         <v>-3.44230914995283</v>
@@ -65072,7 +65077,7 @@
         <v>218.301988527915</v>
       </c>
       <c r="CM226" s="11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="CN226" s="11">
         <v>-2.65542983055935</v>
@@ -65353,7 +65358,7 @@
         <v>208.42005007027799</v>
       </c>
       <c r="CM227" s="11">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="CN227" s="11">
         <v>-6.9511267168716904</v>
@@ -65634,7 +65639,7 @@
         <v>200.904371823579</v>
       </c>
       <c r="CM228" s="11">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="CN228" s="11">
         <v>-7.80706477512277</v>
@@ -65915,7 +65920,7 @@
         <v>181.648551628908</v>
       </c>
       <c r="CM229" s="11">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="CN229" s="11">
         <v>-8.92538855638157</v>
@@ -66196,7 +66201,7 @@
         <v>206.36787235736799</v>
       </c>
       <c r="CM230" s="11">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="CN230" s="11">
         <v>-9.5513572179278992</v>
@@ -66477,7 +66482,7 @@
         <v>280.893373341737</v>
       </c>
       <c r="CM231" s="11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="CN231" s="11">
         <v>-3.8117968789977899</v>
@@ -66758,7 +66763,7 @@
         <v>199.576798755786</v>
       </c>
       <c r="CM232" s="11">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="CN232" s="11">
         <v>-8.2661217602660599</v>
@@ -67039,7 +67044,7 @@
         <v>204.98310252458199</v>
       </c>
       <c r="CM233" s="11">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="CN233" s="11">
         <v>-8.2501605453596696</v>
@@ -67320,7 +67325,7 @@
         <v>235.15131952628701</v>
       </c>
       <c r="CM234" s="11">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="CN234" s="11">
         <v>-5.8508491784398604</v>
@@ -67601,7 +67606,7 @@
         <v>209.65217611233501</v>
       </c>
       <c r="CM235" s="11">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="CN235" s="11">
         <v>-9.2400685409071404</v>
@@ -67882,7 +67887,7 @@
         <v>238.35867223876701</v>
       </c>
       <c r="CM236" s="11">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="CN236" s="11">
         <v>-5.5227574351551798</v>
@@ -68163,7 +68168,7 @@
         <v>213.9366550485</v>
       </c>
       <c r="CM237" s="11">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="CN237" s="11">
         <v>-8.7352863584215008</v>
@@ -68444,7 +68449,7 @@
         <v>258.71117656688301</v>
       </c>
       <c r="CM238" s="11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="CN238" s="11">
         <v>-4.6066698983973797</v>
@@ -68725,7 +68730,7 @@
         <v>237.97977786596999</v>
       </c>
       <c r="CM239" s="11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="CN239" s="11">
         <v>-3.35177217985389</v>
@@ -69006,7 +69011,7 @@
         <v>210.64325938454101</v>
       </c>
       <c r="CM240" s="11">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="CN240" s="11">
         <v>-6.4731377354045998</v>
@@ -69568,7 +69573,7 @@
         <v>205.72842114155901</v>
       </c>
       <c r="CM242" s="11">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="CN242" s="11">
         <v>-7.3667362235481102</v>

</xml_diff>